<commit_message>
Refine utilities workflow and toast notifications
</commit_message>
<xml_diff>
--- a/Cuentas Bancarias NO MOVER.xlsx
+++ b/Cuentas Bancarias NO MOVER.xlsx
@@ -457,22 +457,22 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Empresa</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Banco</t>
+          <t>Bank</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ultimos 4 digitos</t>
+          <t>Last 4 digits</t>
         </is>
       </c>
     </row>

</xml_diff>